<commit_message>
Aplicação completa e em produção
</commit_message>
<xml_diff>
--- a/Planilhas/pedidos_registrados.xlsx
+++ b/Planilhas/pedidos_registrados.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro\Downloads\Program\Planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro\Downloads\PedroDEV\GERENCIADOR DE ROUPAS\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C58905-A32B-4C01-99B9-45F70D23EC82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B1B1A23-F274-4EC1-85E5-17464FC2C0AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>NOME COLABORADOR</t>
   </si>
@@ -40,34 +40,7 @@
     <t>TERMO ASSINADO</t>
   </si>
   <si>
-    <t>MASCULINO</t>
-  </si>
-  <si>
-    <t>PP</t>
-  </si>
-  <si>
-    <t>16/03/2026</t>
-  </si>
-  <si>
-    <t>SIM</t>
-  </si>
-  <si>
-    <t>FEMININO</t>
-  </si>
-  <si>
-    <t>17/03/2026</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>Henrique</t>
-  </si>
-  <si>
-    <t>Flávia</t>
-  </si>
-  <si>
-    <t>Wesley</t>
+    <t>ENTREGA</t>
   </si>
 </sst>
 </file>
@@ -85,7 +58,10 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -146,9 +122,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -186,7 +162,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -220,6 +196,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -254,9 +231,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -430,10 +408,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -452,68 +430,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4">
-        <v>3</v>
-      </c>
-      <c r="E4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>